<commit_message>
Add sign and separation results to the workbook; flip separation criterion to predict-under (|pred| <= |actual|)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -15,7 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Metal Pair" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zhang Comparison" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods and Models" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign and Separation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -621,6 +622,166 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Native classifiers at the Zhang-style cut points (distribution coefficient 0.5 and 10) and a binary logD greater than 0 screen, each with a confidence score (the max class probability). Selective accuracy rises with confidence, which a single flat accuracy does not show. Zhang reference: 3-class accuracy 0.72, macro-F1 0.67.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Macro-F1 or AUC</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Top 25% conf accuracy</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Top 10% conf accuracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Track A new-molecule (Zhang analog)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>3-class</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.912</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Track A new-molecule (Zhang analog)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>binary logD&gt;0</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.742</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.8169999999999999</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.896</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.962</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Track B known-molecule</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>3-class</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.753</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.752</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.956</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.983</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Track B known-molecule</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>binary logD&gt;0</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.973</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.982</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4682,150 +4843,238 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Native classifiers at the Zhang-style cut points (distribution coefficient 0.5 and 10) and a binary logD greater than 0 screen, each with a confidence score (the max class probability). Selective accuracy rises with confidence, which a single flat accuracy does not show. Zhang reference: 3-class accuracy 0.72, macro-F1 0.67.</t>
+          <t>Sign correctness is the fraction where predicted logD has the same sign as actual (extract or not). Separation compares predicted versus actual logD difference between two metals at the same conditions. The predict-under rate is how often the predicted separation magnitude is at most the actual one, meaning the model is conservative about selectivity.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>Track</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Macro-F1 or AUC</t>
+          <t>Top 25% conf</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Top 25% conf accuracy</t>
+          <t>Top 10% conf</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Top 10% conf accuracy</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Track A new-molecule (Zhang analog)</t>
+          <t>Sign correctness (predicted logD sign matches actual)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>3-class</t>
+          <t>A (new molecule)</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.625</v>
+        <v>0.743</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.619</v>
+        <v>0.855</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.854</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>0.912</v>
+        <v>0.903</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Does the model get extract-or-not (logD greater than 0) right</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Track A new-molecule (Zhang analog)</t>
+          <t>Sign correctness</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>binary logD&gt;0</t>
+          <t>B (known molecule)</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.742</v>
+        <v>0.836</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.913</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.896</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>0.962</v>
-      </c>
+        <v>0.919</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Track B known-molecule</t>
+          <t>Separation, signed R2 of the logD difference</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>3-class</t>
+          <t>B (known molecule)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.753</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>0.752</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>0.956</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0.983</v>
+        <v>0.582</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>RMSE 1.069; 44894 metal pairs at matched conditions</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Track B known-molecule</t>
+          <t>Separation, R2 of the magnitude of the difference</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>binary logD&gt;0</t>
+          <t>B (known molecule)</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.832</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>0.973</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>0.982</v>
+        <v>0.312</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>how well the size of the gap is predicted</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Separation, selectivity direction correct</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>B (known molecule)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>picks the right metal as the more extracted one</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Separation, predict-under rate (pred magnitude at most actual)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>B (known molecule)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>the model is conservative, so the real gap is usually at least the predicted one</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Separation, R2 of the magnitude of the difference</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>A (new molecule)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>-0.108</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>RMSE 1.145; new-molecule separation does not predict well, worse than guessing the mean</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Separation, predict-under rate (pred magnitude at most actual)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>A (new molecule)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>conservative overall, but the most confident pairs over-predict more often</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add UCB active-analysis (script, results, workbook sheet)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods and Models" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign and Separation" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -782,6 +783,316 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ranking candidate combinations to test. UCB is the upper end of the 90 percent conformal interval (prediction plus uncertainty). For one-shot screening, ranking by the plain prediction (greedy) finds the strongest extractants and beats UCB, because the uncertainty bonus pulls in uncertain but mediocre candidates. UCB's role is sequential active learning, where exploring uncertain candidates improves the model over rounds. The top 5 percent by prediction reach mean actual logD near 2.2 (new) to 2.6 (known) against 0.02 over all rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Select top %</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Mean actual logD</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Recall of true-best</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>UCB (hi90)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>greedy (prediction)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>UCB (hi90)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>greedy (prediction)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>UCB (hi90)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>greedy (prediction)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.57</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>UCB (hi90)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>greedy (prediction)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add Decision Log sheet documenting every choice and why
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -16,8 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zhang Comparison" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods and Models" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign and Separation" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -629,6 +630,273 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Every major modeling choice and the reason for it, so the project is documented as it evolved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>What we chose</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Two prediction tasks</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Separate new-molecule (A) from known-molecule (B)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Mixing them lets a molecule leak across train and test and inflates the score; an earlier single split read 0.60 and did not hold up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Evaluation</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Molecule-grouped CV for A, random-row CV for B</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Each matches a real use case (screen a new extractant vs tune a known one) without leakage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Data cleaning</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Drop exact duplicates and replicate groups disagreeing by more than 2 log units</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Contradictory labels are noise; cleaning took 8075 rows to 7065.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Track A model</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Single tuned LightGBM</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>The stack adds accuracy but makes residuals less rankable, which weakens confidence; the single model ranks confidence better for screening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Track B model</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>NNLS stack of trees (ExtraTrees, LightGBM, XGBoost, CatBoost)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Stacking improves both accuracy and confidence here, and NNLS sets weak members to zero on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>A: conditions + metal; B: also ECFP + ligand</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Structure does not generalize from about 300 molecules (A); it helps once the molecule has been seen (B). RDKit blocks and embeddings did not beat ECFP plus conditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>err_lgb on plain features, ranked; normalized split-conformal intervals</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Richer features (member predictions, disagreement, novelty) ranked worse; the intervals hit their target coverage (0.89 to 0.90).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Graph network</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Chemprop alone reached only R2 0.23 on new molecules and added nothing when blended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>TabPFN</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>As a local expert it earned only 0.13 NNLS weight and +0.0011 R2, with error-correlation 0.82 to the trees (not diverse).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Hyperparameter search</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Kept near-default settings</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>A randomized search moved Track A 0.466 to 0.484 and Track B not at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Separation criterion</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Predict-under: predicted gap at most the actual gap</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Direction does not matter since the other metal stays in solution for a known extractant; a conservative predicted gap means the real gap is at least as large.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Active analysis</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Rank by prediction for one-shot screening; UCB for sequential rounds</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>UCB's uncertainty bonus pulls in mediocre candidates, so greedy finds the strongest now; UCB pays off only when exploring to improve the model over rounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Comparison with Dr. Zhang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Same 8075-row dataset, scored on his split</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Our model matches his accuracy on his own test; the added value is continuous logD with calibrated confidence rather than one of three buckets.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -783,7 +1051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add sequential active-learning UCB experiment (script, results, figure, workbook sheet)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active learning (sequential)" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1361,6 +1362,104 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sequential active learning: each round picks the next batch to run, reveals logD, and retrains. For finding strong extractants (discovery) greedy and UCB win, about 0.72 of the true best found. For improving the model (test R2) uncertainty sampling wins at 0.56, while greedy and UCB hurt it by over-sampling the high-logD region and biasing the training set. UCB tracks greedy here, so the best acquisition depends on whether the goal is discovery or model improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Final test R2 (model quality)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Final discovery (share of true top-10% found)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.347</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>greedy</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.728</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ucb</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.713</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.5610000000000001</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.383</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add experiment triage: trust confident predictions, test the uncertain ones
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active learning (sequential)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment triage" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1460,6 +1461,214 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The high-confidence predictions do not need experiments; they are trusted as-is, so the experiment budget goes to the uncertain remainder. For known molecules the most confident half can be accepted at RMSE 0.535 with 75 percent within half a log unit, which halves the experiments needed. New molecules degrade faster, so a smaller, more confident slice is accepted. For the experiments that are run, sampling by uncertainty improves the model fastest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Auto-accept most confident %</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Experiments saved</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Experiments still needed</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Accepted RMSE</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Accepted within 0.5 log units</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>5298</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>3535</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>3530</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>59%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Track A (new molecule)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>5299</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1766</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>51%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>5298</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>3535</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>3530</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Track B (known molecule)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>5299</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1766</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.631</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>67%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add confidence-algorithm acquisition to active-learning comparison
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -1369,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1380,7 +1380,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sequential active learning: each round picks the next batch to run, reveals logD, and retrains. For finding strong extractants (discovery) greedy and UCB win, about 0.72 of the true best found. For improving the model (test R2) uncertainty sampling wins at 0.56, while greedy and UCB hurt it by over-sampling the high-logD region and biasing the training set. UCB tracks greedy here, so the best acquisition depends on whether the goal is discovery or model improvement.</t>
+          <t>Sequential active learning: each round picks the next batch to run, reveals logD, and retrains. For finding strong extractants (discovery) greedy and UCB win, about 0.72 of the true best found. For improving the model (test R2) the ensemble-disagreement uncertainty wins at 0.56. Acquiring by the confidence algorithm's own predicted error, the same err model used to decide which predictions to trust, helps discovery (0.44) but improves the model less (0.465), because large predicted error flags the hard, extreme-logD points rather than under-sampled regions, which biases the training set much as greedy does. So the err model is the right tool for deciding which predictions to trust, while ensemble disagreement is the right signal for choosing points that most improve the model.</t>
         </is>
       </c>
     </row>
@@ -1451,6 +1451,19 @@
       </c>
       <c r="C6" s="3" t="n">
         <v>0.383</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add ECM free-energy model: delta G target, conditions dropped, per-row vs per-pair
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active learning (sequential)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment triage" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECM (free energy target)" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1682,6 +1683,126 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ECM predicts the Gibbs free energy of extraction (delta G = -2.303 R T logD, in kJ/mol, so favorable extraction is negative) from the extractant structure and the metal, with all reaction conditions dropped. Per-row keeps every measurement; per-pair averages delta G to one value per extractant-metal-acid-diluent system and is condition-independent. Per-pair is the better target (R2 0.42 versus 0.27) because identical structures otherwise repeat with condition-driven delta G the structure cannot explain. Confidence ranking is strong for per-pair: the most confident quarter reach R2 0.68 and the top tenth R2 0.81 (RMSE 3.2 kJ/mol). Molecule-grouped cross-validation, so a new extractant never appears in both train and test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Framing</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Systems</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>R2 all</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>RMSE all (kJ/mol)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>R2 top 25% conf</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>R2 top 10% conf</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>RMSE top 10% (kJ/mol)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>per-row (framing 1)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>7066</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.515</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>5.22</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>per-pair (framing 3)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2273</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>3.24</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
ECM ensemble sweep: RandomForest is best (R2 0.473), stack only ties; switch ECM to RandomForest, add sweep sheet and slide, update docs
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -22,6 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active learning (sequential)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment triage" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECM (free energy target)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECM ensemble sweep" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1704,7 +1705,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ECM predicts the Gibbs free energy of extraction (delta G = -2.303 R T logD, in kJ/mol, so favorable extraction is negative) from the extractant structure and the metal, with all reaction conditions dropped. Per-row keeps every measurement; per-pair averages delta G to one value per extractant-metal-acid-diluent system and is condition-independent. Per-pair is the better target (R2 0.42 versus 0.27) because identical structures otherwise repeat with condition-driven delta G the structure cannot explain. Confidence ranking is strong for per-pair: the most confident quarter reach R2 0.68 and the top tenth R2 0.81 (RMSE 3.2 kJ/mol). Molecule-grouped cross-validation, so a new extractant never appears in both train and test.</t>
+          <t>ECM predicts the Gibbs free energy of extraction (delta G = -2.303 R T logD, in kJ/mol, so favorable extraction is negative) from the extractant structure and the metal, with all reaction conditions dropped. The model is a RandomForest, the best of an ensemble sweep (see the ECM ensemble sweep sheet). Per-row keeps every measurement; per-pair averages delta G to one value per extractant-metal-acid-diluent system and is condition-independent. Per-pair is the better target (R2 0.47 versus 0.28) because identical structures otherwise repeat with condition-driven delta G the structure cannot explain. Confidence ranking is strong for per-pair: the most confident quarter reach R2 0.68 and the top tenth R2 0.78 (RMSE 3.6 kJ/mol). Molecule-grouped cross-validation, so a new extractant never appears in both train and test.</t>
         </is>
       </c>
     </row>
@@ -1755,19 +1756,19 @@
         <v>7066</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.27</v>
+        <v>0.282</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>7.62</v>
+        <v>7.55</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.48</v>
+        <v>0.404</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.515</v>
+        <v>0.518</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>5.22</v>
+        <v>4.85</v>
       </c>
     </row>
     <row r="4">
@@ -1780,24 +1781,200 @@
         <v>2273</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.424</v>
+        <v>0.473</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>6.6</v>
+        <v>6.31</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.678</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.776</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>3.24</v>
+        <v>3.62</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ensemble sweep for the per-pair delta G target: each base model under molecule-grouped cross-validation, then equal-weight and NNLS stacks. RandomForest is the best single model (R2 0.473), with the bagged-tree models ahead of the boosters on this small wide table and Ridge near zero (the signal is nonlinear). The NNLS stack, scored with a second cross-validation (0.474), only ties RandomForest, so stacking adds nothing here and the ECM uses plain RandomForest. NNLS weights: RandomForest 0.56, CatBoost 0.28, ExtraTrees 0.19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>R2 (per-pair dG)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>RMSE (kJ/mol)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>LightGBM</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>ExtraTrees</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>6.62</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.473</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>6.31</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>HistGB</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>6.58</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>8.58</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>6.48</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CatBoost</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>equal-weight</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>NNLS stack (in-sample)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>6.28</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>NNLS stack (CV)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>6.31</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Run UCB active analysis and pseudo-labeling on the delta G model
UCB on dG: greedy best for one-shot, triage accepts confident quarter.
Pseudo-labeling confident predictions barely helps (+0.00 to +0.01 R2);
oracle with true labels helps (+0.06 to +0.10), so experiments add the info.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -23,6 +23,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment triage" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECM (free energy target)" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECM ensemble sweep" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G UCB" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G pseudo-labeling" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1980,6 +1982,364 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>UCB active analysis run on the delta G model, since delta G is the predictor that drives the screening. To find the strongest extractants (most negative delta G), ranking by the plain prediction (greedy) is best for a one-shot pick: the top 5 percent average delta G -10.5 kJ/mol versus -0.3 at random, while UCB's uncertainty term dilutes that and is for sequential rounds. Triage: the most confident quarter of predictions can be accepted without experiments at RMSE about 4 kJ/mol, so the experiment budget goes to the uncertain rest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Top %</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Mean actual dG / RMSE (kJ/mol)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Recall / within 3 kJ/mol</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>UCB selection</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>UCB (pred - unc)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>-4.13</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>UCB selection</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>greedy (pred)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>-10.47</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>UCB selection</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>UCB selection</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>UCB (pred - unc)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>-4.06</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>UCB selection</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>greedy (pred)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>-8.539999999999999</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>UCB selection</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>triage</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>accept confident</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>triage</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>accept confident</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.54</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Testing the idea of adding confident predictions (the narrow 90 percent interval ones) as training rows without experiments. Adding the model's own confident predictions barely helps (test R2 +0.00 to +0.01), because a confident prediction carries no new information. Adding the same systems with their true labels, which is what running the experiments would give, helps materially (+0.06 to +0.10). So confidence is for deciding which predictions to trust and skip, not for manufacturing training data; the real gains come from experiments on the uncertain points.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Confident added %</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Test R2</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Test RMSE (kJ/mol)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>baseline (seed only)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>7.07</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>pseudo (predicted labels)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>7.06</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>oracle (true labels)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.355</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>6.76</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>pseudo (predicted labels)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>6.99</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>oracle (true labels)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.392</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>6.56</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Rename ECM to the free-energy (delta G) model everywhere
Drop the undefined ECM label across scripts (ecm*.py -> dg_*.py), result
CSVs, the figure, the workbook sheets, the README section, and the slides.
The free-energy model feeds the UCB screening. Re-ran the model and ensemble
scripts to confirm identical numbers (per-pair R2 0.473, RMSE 6.31 kJ/mol).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -21,8 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active learning (sequential)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment triage" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECM (free energy target)" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECM ensemble sweep" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Free energy (delta G)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G ensemble sweep" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G UCB" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G pseudo-labeling" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
@@ -1707,7 +1707,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ECM predicts the Gibbs free energy of extraction (delta G = -2.303 R T logD, in kJ/mol, so favorable extraction is negative) from the extractant structure and the metal, with all reaction conditions dropped. The model is a RandomForest, the best of an ensemble sweep (see the ECM ensemble sweep sheet). Per-row keeps every measurement; per-pair averages delta G to one value per extractant-metal-acid-diluent system and is condition-independent. Per-pair is the better target (R2 0.47 versus 0.28) because identical structures otherwise repeat with condition-driven delta G the structure cannot explain. Confidence ranking is strong for per-pair: the most confident quarter reach R2 0.68 and the top tenth R2 0.78 (RMSE 3.6 kJ/mol). Molecule-grouped cross-validation, so a new extractant never appears in both train and test.</t>
+          <t>The free-energy model predicts the Gibbs free energy of extraction (delta G = -2.303 R T logD, in kJ/mol, so favorable extraction is negative) from the extractant structure and the metal, with all reaction conditions dropped. The model is a RandomForest, the best of an ensemble sweep (see the Delta G ensemble sweep sheet). Per-row keeps every measurement; per-pair averages delta G to one value per extractant-metal-acid-diluent system and is condition-independent. Per-pair is the better target (R2 0.47 versus 0.28) because identical structures otherwise repeat with condition-driven delta G the structure cannot explain. Confidence ranking is strong for per-pair: the most confident quarter reach R2 0.68 and the top tenth R2 0.78 (RMSE 3.6 kJ/mol). Molecule-grouped cross-validation, so a new extractant never appears in both train and test.</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ensemble sweep for the per-pair delta G target: each base model under molecule-grouped cross-validation, then equal-weight and NNLS stacks. RandomForest is the best single model (R2 0.473), with the bagged-tree models ahead of the boosters on this small wide table and Ridge near zero (the signal is nonlinear). The NNLS stack, scored with a second cross-validation (0.474), only ties RandomForest, so stacking adds nothing here and the ECM uses plain RandomForest. NNLS weights: RandomForest 0.56, CatBoost 0.28, ExtraTrees 0.19.</t>
+          <t>Ensemble sweep for the per-pair delta G target: each base model under molecule-grouped cross-validation, then equal-weight and NNLS stacks. RandomForest is the best single model (R2 0.473), with the bagged-tree models ahead of the boosters on this small wide table and Ridge near zero (the signal is nonlinear). The NNLS stack, scored with a second cross-validation (0.474), only ties RandomForest, so stacking adds nothing here and the free-energy model uses plain RandomForest. NNLS weights: RandomForest 0.56, CatBoost 0.28, ExtraTrees 0.19.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add confidence sweeps: confidence curve per model, and a confidence-ranker sweep
Part A: all tree models gain from confidence filtering (top-10% R2 ~0.75-0.79);
XGBoost/HistGB edge RF on the confident sliver, RF best overall, CatBoost worst.
Part B: learned err models (LightGBM/RF) rank confidence best; RF tree-spread
is weakest, validating the LightGBM err model. Also expanded model sweep (TabPFN
guarded on CPU, kNN/SVR/tuned-RF all below RF).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G ensemble sweep" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G UCB" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G pseudo-labeling" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confidence sweep" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2340,6 +2341,310 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Two sweeps on the per-pair delta G model. Part A applies the same LightGBM confidence ranker to each prediction model: all tree models benefit, climbing from about 0.42-0.47 overall to roughly 0.75-0.79 at the most confident tenth, with XGBoost and HistGB edging RandomForest on that small sliver while RandomForest stays best overall, and CatBoost the outlier whose errors are least predictable. Part B fixes the predictor at RandomForest and sweeps the confidence estimator: the learned err models (LightGBM, RandomForest) rank best and are about tied, while RandomForest's own tree-spread is the weakest ranker, which is why a learned err model is used rather than the native uncertainty. The current setup (RandomForest predictor, LightGBM err ranker) is validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Model or ranker</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>All R2</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Top 25% R2</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Top 10% R2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Top 10% RMSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>A pred-model</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.473</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.6889999999999999</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>3.71</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A pred-model</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ExtraTrees</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>4.04</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>A pred-model</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HistGB</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.671</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.785</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>A pred-model</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>LightGBM</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.428</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.6889999999999999</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.753</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>3.84</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>A pred-model</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.789</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>A pred-model</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>CatBoost</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.434</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.602</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>4.02</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>B conf-ranker (RF)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>err-LightGBM</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.473</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.6889999999999999</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>3.71</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>B conf-ranker (RF)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>err-RandomForest</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.473</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.696</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.748</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>3.32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>B conf-ranker (RF)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>err-ExtraTrees</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.473</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>3.73</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>B conf-ranker (RF)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>RF tree-spread (native)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0.473</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Verify delta G interval calibration: 90% covers 90.2%, 80% covers 80.2%
The calibrated, heterogeneous intervals are what make the active analysis work:
trust and skip the confident (narrow-interval) predictions, test the uncertain.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -26,6 +26,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G UCB" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G pseudo-labeling" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confidence sweep" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G interval calibration" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3399,6 +3400,72 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Honest molecule-split conformal check of the delta G prediction intervals: the conformal quantile is set on one set of molecules and coverage is measured on a disjoint set. The 90 percent interval covers 90.2 percent of held-out cases and the 80 percent interval covers 80.2 percent, so the stated confidence can be trusted. The intervals are calibrated and heterogeneous: the confident, narrow-interval predictions are the accurate ones (most confident tenth R2 0.78, RMSE 3.6 kJ/mol), while the uncertain ones get wide intervals and are sent to the lab. This calibration is what lets the intervals drive the active analysis: trust and skip the confident predictions, test the uncertain ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Empirical coverage</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Mean width (kJ/mol)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Audit remediation: honest numbers and framing across README, workbook, slides
Track B logD relabeled (honest ~0.61 condition-key; 0.725 = random-row upper bound
with replicate memorization; ~0.44 on new molecules). delta G headline ~0.46+/-0.01.
Zhang reframed to the same-data comparison (drop the off-dataset 0.605). Added an
Audit corrections workbook tab and slide, the honest logD recompute (track_ab_results.csv),
and the two trend figures/slides.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -8,25 +8,26 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Comparison" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confidence" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Metal" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Metal Pair" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zhang Comparison" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods and Models" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign and Separation" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active learning (sequential)" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment triage" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Free energy (delta G)" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G ensemble sweep" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G UCB" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G pseudo-labeling" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confidence sweep" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G interval calibration" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit corrections" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confidence" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Metal" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Metal Pair" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zhang Comparison" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods and Models" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign and Separation" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifier with Confidence" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active analysis (UCB)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active learning (sequential)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment triage" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Free energy (delta G)" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G ensemble sweep" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G UCB" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G pseudo-labeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confidence sweep" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delta G interval calibration" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -638,6 +639,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sign correctness is the fraction where predicted logD has the same sign as actual (extract or not). Separation compares predicted versus actual logD difference between two metals at the same conditions. The predict-under rate is how often the predicted separation magnitude is at most the actual one, meaning the model is conservative about selectivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Top 25% conf</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Top 10% conf</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Sign correctness (predicted logD sign matches actual)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>A (new molecule)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Does the model get extract-or-not (logD greater than 0) right</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Sign correctness</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>B (known molecule)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.836</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.913</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Separation, signed R2 of the logD difference</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>B (known molecule)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>RMSE 1.069; 44894 metal pairs at matched conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Separation, R2 of the magnitude of the difference</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>B (known molecule)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>how well the size of the gap is predicted</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Separation, selectivity direction correct</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>B (known molecule)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>picks the right metal as the more extracted one</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Separation, predict-under rate (pred magnitude at most actual)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>B (known molecule)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>the model is conservative, so the real gap is usually at least the predicted one</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Separation, R2 of the magnitude of the difference</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>A (new molecule)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>-0.108</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>RMSE 1.145; new-molecule separation does not predict well, worse than guessing the mean</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Separation, predict-under rate (pred magnitude at most actual)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>A (new molecule)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>conservative overall, but the most confident pairs over-predict more often</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -899,7 +1148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1059,7 +1308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1369,7 +1618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1480,7 +1729,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1688,7 +1937,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1808,7 +2057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1984,7 +2233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2210,7 +2459,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2342,7 +2591,235 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Corrections from a full adversarial audit. The modeling is fundamentally honest: genuine molecule-grouped cross-validation with zero train/test molecule overlap, no feature encodes the target, and the confidence intervals are calibrated (90 percent covers 90 percent). These entries correct optimistic framing and the Track B replicate-memorization leakage so the reported numbers match what the evaluation supports. Where other sheets still show the earlier values, this sheet supersedes them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Honest value</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Previously reported</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Why / caveat</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Track A new-molecule logD R2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>0.466 (RMSE 1.148)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>0.466</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Honest, molecule-grouped CV. Unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Track B logD R2 (honest)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>about 0.61 (RMSE about 0.98)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0.725</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>0.725 used a random-row split that memorizes replicate siblings (the fingerprint is constant within a molecule); about 0.07 R2 is leakage. The honest 0.61 is condition-key grouped: interpolate new conditions for an already-seen molecule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Track B on NEW molecules</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>about 0.44</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>read as 0.725</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>The rich features collapse to about Track A on unseen molecules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>delta G per-pair R2</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>0.46 plus or minus 0.01 (RMSE 6.3)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0.473</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>0.473 was the maximum of a roughly 55-way model and hyperparameter search on one fixed split; the mean over shuffled molecule-grouped splits is 0.461 plus or minus 0.009.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Top-10 percent confidence R2</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>selective-prediction operating point</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0.912 / 0.940 / 0.776</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Report the RMSE drop; the R2 rise is partly the shrinking variance of the retained subset. The Track B 0.940 is on a leaky split and is being recomputed on the condition-key split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Zhang comparison</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>ours 0.657 CV / 0.692 holdout vs his 0.648 / 0.680</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>his 0.605; we match 0.72</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>0.605 was his model run on our data on a different split, which widened the gap. The same-data comparison shows the models about equal, so the split, not the model, drives his 0.72 headline. His 0.72 reproduces at 0.68; ours is 0.692 on his holdout (within 0.03).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Per-metal and classifier R2</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>known-molecule (random CV) values</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0.80+ per metal; 0.753 classifier</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>These are known-molecule optimistic. The grouped classifier is 0.625 (3-class) vs a 0.385 majority baseline; the per-metal new-molecule numbers are lower.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Data basis</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>label-QC-cleaned (8075 to 7066 rows); noise floor about 0.45 log units</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>across all rows</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Cleaning (replicate logD range at most 2) also removes the hardest measurements from evaluation, so all absolute numbers are an upper bound.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2646,7 +3123,73 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Honest molecule-split conformal check of the delta G prediction intervals: the conformal quantile is set on one set of molecules and coverage is measured on a disjoint set. The 90 percent interval covers 90.2 percent of held-out cases and the 80 percent interval covers 80.2 percent, so the stated confidence can be trusted. The intervals are calibrated and heterogeneous: the confident, narrow-interval predictions are the accurate ones (most confident tenth R2 0.78, RMSE 3.6 kJ/mol), while the uncertain ones get wide intervals and are sent to the lab. This calibration is what lets the intervals drive the active analysis: trust and skip the confident predictions, test the uncertain ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Empirical coverage</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Mean width (kJ/mol)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3400,73 +3943,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Honest molecule-split conformal check of the delta G prediction intervals: the conformal quantile is set on one set of molecules and coverage is measured on a disjoint set. The 90 percent interval covers 90.2 percent of held-out cases and the 80 percent interval covers 80.2 percent, so the stated confidence can be trusted. The intervals are calibrated and heterogeneous: the confident, narrow-interval predictions are the accurate ones (most confident tenth R2 0.78, RMSE 3.6 kJ/mol), while the uncertain ones get wide intervals and are sent to the lab. This calibration is what lets the intervals drive the active analysis: trust and skip the confident predictions, test the uncertain ones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Empirical coverage</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Mean width (kJ/mol)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>0.902</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>0.802</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3829,7 +4306,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4286,7 +4763,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4906,7 +5383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6294,7 +6771,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6539,7 +7016,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>His XGBoost under our cross-validation</t>
+          <t>His XGBoost, same-data comparison</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -6549,7 +7026,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>0.605 over all new molecules; same model on honest CV, so 0.72 reflects the favorable holdout and the imbalanced classes, not a stronger model</t>
+          <t>On the same data his model scores 0.648 (our CV) and 0.680 (his holdout); his 0.72 reproduces at 0.68. The split, not a stronger model, drives the headline. An earlier 0.605 figure was his model on a different split and overstated the gap.</t>
         </is>
       </c>
     </row>
@@ -6583,7 +7060,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>0.692 raw, which matches him; with our confidence 0.863 at top 25 percent and 1.000 at top 10 percent; also returns continuous logD (R2 0.360) and an interval</t>
+          <t>0.692, within about 0.03 of his 0.72; with our confidence 0.863 at top 25 percent and 1.000 at top 10 percent; also returns continuous logD (R2 0.360) and an interval</t>
         </is>
       </c>
     </row>
@@ -6617,7 +7094,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Matches on new molecules once confidence is used (0.912 at top 10 percent), beats 0.72 outright on known molecules (0.753), and also returns the value, the uncertainty, and the separations</t>
+          <t>About equal on the same-data common split (0.657 vs 0.648 our CV; 0.692 vs 0.680 his holdout), so the split drives his headline. Our added value is calibrated uncertainty, continuous logD, and the separations, not higher accuracy.</t>
         </is>
       </c>
     </row>
@@ -6629,7 +7106,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6765,252 +7242,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Sign correctness is the fraction where predicted logD has the same sign as actual (extract or not). Separation compares predicted versus actual logD difference between two metals at the same conditions. The predict-under rate is how often the predicted separation magnitude is at most the actual one, meaning the model is conservative about selectivity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Analysis</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Track</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Top 25% conf</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Top 10% conf</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Sign correctness (predicted logD sign matches actual)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>A (new molecule)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>0.743</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>0.855</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0.903</v>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Does the model get extract-or-not (logD greater than 0) right</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Sign correctness</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>B (known molecule)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0.836</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0.913</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>0.919</v>
-      </c>
-      <c r="F4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Separation, signed R2 of the logD difference</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>B (known molecule)</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.582</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>RMSE 1.069; 44894 metal pairs at matched conditions</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Separation, R2 of the magnitude of the difference</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>B (known molecule)</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>0.312</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>how well the size of the gap is predicted</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Separation, selectivity direction correct</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>B (known molecule)</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>0.763</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>picks the right metal as the more extracted one</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Separation, predict-under rate (pred magnitude at most actual)</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>B (known molecule)</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>0.633</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>the model is conservative, so the real gap is usually at least the predicted one</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Separation, R2 of the magnitude of the difference</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>A (new molecule)</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>-0.108</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>RMSE 1.145; new-molecule separation does not predict well, worse than guessing the mean</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Separation, predict-under rate (pred magnitude at most actual)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>A (new molecule)</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>0.5669999999999999</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>0.541</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>conservative overall, but the most confident pairs over-predict more often</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix .gitignore conflict markers; recompute the Track B confidence curve on the condition-key split (honest top-10% R2 0.874, RMSE 0.430); propagate the honest numbers into the deck, workbook, README, and methods doc
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Report the RMSE drop; the R2 rise is partly the shrinking variance of the retained subset. The Track B 0.940 is on a leaky split and is being recomputed on the condition-key split.</t>
+          <t>Report the RMSE drop; the R2 rise is partly the shrinking variance of the retained subset. The Track B 0.940 was on a leaky split; recomputed on the condition-key split it is 0.874 (RMSE 0.430), with all-rows R2 0.611.</t>
         </is>
       </c>
     </row>
@@ -7187,7 +7187,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>A second model (err_lgb) predicts the absolute error of each prediction from the conditions and the prediction. Rows are ranked by predicted error. The top 10 to 25 percent by confidence are much more accurate (Track B top 10% R2 0.940, RMSE 0.341).</t>
+          <t>A second model (err_lgb) predicts the absolute error of each prediction from the conditions and the prediction. Rows are ranked by predicted error. The top 10 to 25 percent by confidence are much more accurate (honest condition-key Track B top 10% R2 0.874, RMSE 0.430; the earlier 0.940 was on a leaky random-row split).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply final-audit fixes (model-agnostic confidence framing for Zhang, reproducible verification script for the gap-bin/bootstrap/random-rank controls, 23-vs-28 element count, per-pair confidence scoped to RMSE), confirm end-to-end reproducibility from data.zip, and add the manuscript figure/table bundle
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REE_Results_Organized.xlsx
+++ b/docs/REE_Results_Organized.xlsx
@@ -5242,7 +5242,7 @@
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>This is the audited honest dG headline (~0.46-0.47). An earlier 0.473 framing figure is consistent here; do not regress to inflated numbers.</t>
+          <t>The audited honest dG headline is R2 ~0.461 +/- 0.009; the 0.473 in the Value cell is the selected maximum of a ~55-way search, not the headline. Do not regress to inflated numbers.</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
@@ -10957,7 +10957,7 @@
       </c>
       <c r="L131" s="5" t="inlineStr">
         <is>
-          <t>sep_factor_confidence.py: applies the err-model confidence layer (our differentiator) to separation; the most-confident 10% reaches direction 0.789 and normalized RMSE 0.64, beating random-rank 0.80, showing confidence-filtered separation calls are trustworthy for known extractants</t>
+          <t>sep_factor_confidence.py applies the err-model confidence layer (our differentiator) to separation; the most-confident 10% reaches direction 0.789 and normalized RMSE (RMSE/spread) 0.64, which beats a random-ranking benchmark of 0.80 (the gap-bin, bootstrap, and random-rank controls are computed in sep_factor_confidence_verify.py).</t>
         </is>
       </c>
       <c r="M131" s="5" t="inlineStr">
@@ -11818,7 +11818,7 @@
       </c>
       <c r="J144" s="5" t="inlineStr">
         <is>
-          <t>each pair has mean_conf_err; high-err pairs systematically coincide with poor/negative sep_R2</t>
+          <t>each pair has mean_conf_err; it tracks separation RMSE (Spearman ~0.73) but is roughly uninformative about skill-based separation R2 (Spearman ~-0.11).</t>
         </is>
       </c>
       <c r="K144" s="5" t="inlineStr">
@@ -11828,7 +11828,7 @@
       </c>
       <c r="L144" s="5" t="inlineStr">
         <is>
-          <t>Per the rules, the large per-pair table is summarized rather than enumerated; the pattern across all 70 is that mean_conf_err is inversely related to separation quality, which is the project's core claim that the confidence layer flags unreliable separations.</t>
+          <t>Per the rules, the large per-pair table is summarized rather than enumerated; across all 70 pairs mean_conf_err tracks separation RMSE (Spearman ~0.73) but not skill-based R2 (Spearman ~-0.11), so confidence flags high-error pairs rather than ranking separation skill.</t>
         </is>
       </c>
       <c r="M144" s="5" t="inlineStr">
@@ -16675,7 +16675,7 @@
       </c>
       <c r="J223" s="5" t="inlineStr">
         <is>
-          <t>Zhang has NO confidence layer; cannot reach our confidence-filtered direction 0.789</t>
+          <t>Our model-agnostic confidence layer, applied to his predictions, lifts his known top-10% signed R2 0.369 to 0.470 (direction 0.704); our model reaches 0.591 (direction 0.789). His published model includes no confidence ranking.</t>
         </is>
       </c>
       <c r="K223" s="5" t="inlineStr">
@@ -16685,7 +16685,7 @@
       </c>
       <c r="L223" s="5" t="inlineStr">
         <is>
-          <t>sep_factor_zhang.py: reimplements Dr. Zhang's XGBoost+ECFP and differences it the same way; it ties our point model (0.369 vs 0.356, dir 0.715 vs 0.726), but because it has no confidence layer it cannot reach our confidence-filtered direction 0.789, which is the project's differentiator</t>
+          <t>sep_factor_zhang.py reimplements Dr. Zhang's XGBoost+ECFP and differences it the same way; it ties our point model on known extractants (0.369 vs 0.356, direction 0.715 vs 0.726). The confidence layer is our model-agnostic addition: applied to his predictions his most-confident tenth still trails ours (direction 0.704 vs 0.789).</t>
         </is>
       </c>
       <c r="M223" s="5" t="inlineStr">
@@ -16742,7 +16742,7 @@
       </c>
       <c r="J224" s="5" t="inlineStr">
         <is>
-          <t>no confidence layer</t>
+          <t>Confidence layer applied to his predictions: top-10% signed R2 0.140, no improvement; for new extractants confidence does not help either model.</t>
         </is>
       </c>
       <c r="K224" s="5" t="inlineStr">
@@ -16982,7 +16982,7 @@
       </c>
       <c r="J228" s="5" t="inlineStr">
         <is>
-          <t>none (Zhang's model has no confidence layer; that gap is exactly what this project adds)</t>
+          <t>Zhang's published model includes no confidence ranking; our model-agnostic confidence layer is what this project adds, and it can wrap either base model.</t>
         </is>
       </c>
       <c r="K228" s="5" t="inlineStr">

</xml_diff>